<commit_message>
Enhance date handling in WbsWorkbook and MainFrame
- Updated WbsWorkbook to improve date parsing for numeric and formula cells, allowing for better handling of Excel date formats.
- Refactored date handling in MainFrame to utilize LocalDate directly, simplifying date manipulation and improving clarity.
- Introduced custom spinner model and editor for date selection in the UI.
- Added unit test to verify reading of numeric and formula date headers without explicit date formatting in Excel.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n-sug.INSPIRON5515\Desktop\github\excel-edit-java\"/>
     </mc:Choice>
@@ -15,10 +15,10 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
   <si>
     <t>WBS No</t>
     <phoneticPr fontId="1"/>
@@ -109,12 +109,19 @@
       <t>ショウコウモク</t>
     </rPh>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>10月1日</t>
+  </si>
+  <si>
+    <t>木</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -443,137 +450,153 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:L11"/>
+  <dimension ref="A2:M11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" style="1"/>
-    <col min="6" max="12" width="8" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="6.0"/>
+    <col min="2" max="2" style="1" width="9.0"/>
+    <col min="6" max="6" customWidth="true" width="12.0"/>
+    <col min="7" max="7" customWidth="true" width="8.0"/>
+    <col min="8" max="8" customWidth="true" width="8.0"/>
+    <col min="9" max="9" customWidth="true" width="8.0"/>
+    <col min="10" max="10" customWidth="true" width="8.0"/>
+    <col min="11" max="11" customWidth="true" width="8.0"/>
+    <col min="12" max="12" customWidth="true" width="8.0"/>
+    <col min="13" max="13" customWidth="true" width="8.0"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:12">
-      <c r="F2" s="3">
+      <c r="F2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3">
         <v>46296</v>
       </c>
-      <c r="G2" s="3">
-        <f t="shared" ref="G2:L2" si="0">F2+1</f>
-        <v>46297</v>
-      </c>
-      <c r="H2" s="3">
+      <c r="H2" s="3" t="n">
+        <f t="shared" ref="H2:M2" si="0">G2+1</f>
+        <v>46297.0</v>
+      </c>
+      <c r="I2" s="3" t="n">
         <f t="shared" si="0"/>
-        <v>46298</v>
-      </c>
-      <c r="I2" s="3">
+        <v>46298.0</v>
+      </c>
+      <c r="J2" s="3" t="n">
         <f t="shared" si="0"/>
-        <v>46299</v>
-      </c>
-      <c r="J2" s="3">
+        <v>46299.0</v>
+      </c>
+      <c r="K2" s="3" t="n">
         <f t="shared" si="0"/>
-        <v>46300</v>
-      </c>
-      <c r="K2" s="3">
+        <v>46300.0</v>
+      </c>
+      <c r="L2" s="3" t="n">
         <f t="shared" si="0"/>
-        <v>46301</v>
-      </c>
-      <c r="L2" s="3">
+        <v>46301.0</v>
+      </c>
+      <c r="M2" s="3" t="n">
         <f t="shared" si="0"/>
-        <v>46302</v>
+        <v>46302.0</v>
       </c>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="F3" t="str">
-        <f>TEXT(F2,"aaa")</f>
+      <c r="F3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="G3" t="str" s="0">
+        <f>TEXT(G2,"aaa")</f>
         <v>木</v>
       </c>
-      <c r="G3" t="str">
-        <f t="shared" ref="G3:L3" si="1">TEXT(G2,"aaa")</f>
+      <c r="H3" t="str" s="0">
+        <f t="shared" ref="H3:M3" si="1">TEXT(H2,"aaa")</f>
         <v>金</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str" s="0">
         <f t="shared" si="1"/>
         <v>土</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str" s="0">
         <f t="shared" si="1"/>
         <v>日</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str" s="0">
         <f t="shared" si="1"/>
         <v>月</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str" s="0">
         <f t="shared" si="1"/>
         <v>火</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str" s="0">
         <f t="shared" si="1"/>
         <v>水</v>
       </c>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4">
+      <c r="A4" s="0">
         <v>1</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="D5" s="2"/>
-      <c r="E5" t="s">
+      <c r="E5" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6">
+      <c r="A6" s="0">
         <v>2</v>
       </c>
       <c r="B6" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="D7" s="2"/>
-      <c r="E7" t="s">
+      <c r="E7" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8">
+      <c r="A8" s="0">
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" t="s" s="0">
         <v>7</v>
+      </c>
+      <c r="J8" t="n" s="0">
+        <v>1.0</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -581,28 +604,34 @@
         <f>D8</f>
         <v>菅原</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="I9">
-        <v>2.5</v>
+      <c r="F9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="J9" t="n" s="0">
+        <v>1.5</v>
       </c>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10">
+      <c r="A10" s="0">
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" t="s" s="0">
         <v>7</v>
+      </c>
+      <c r="J10" t="n" s="0">
+        <v>2.0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -610,11 +639,14 @@
         <f>D10</f>
         <v>菅原</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="I11">
-        <v>1.5</v>
+      <c r="F11" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="J11" t="n" s="0">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor hours formatting and enhance cell editing in MainFrame
- Updated Hours class to format decimal values consistently with two decimal places.
- Introduced a new CellStyle for hours in WbsWorkbook to ensure proper formatting in Excel.
- Enhanced MainFrame's HoursEditor to support overwriting text on key input, improving user experience.
- Added unit tests to verify formatting changes and cell style application in Excel.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -165,11 +165,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="56" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -610,8 +611,8 @@
       <c r="F9" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="J9" t="n" s="0">
-        <v>1.5</v>
+      <c r="J9" t="n" s="4">
+        <v>3.0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -645,8 +646,8 @@
       <c r="F11" t="n" s="0">
         <v>2.0</v>
       </c>
-      <c r="J11" t="n" s="0">
-        <v>2.5</v>
+      <c r="J11" t="n" s="4">
+        <v>4.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance WbsWorkbook with calculation chain management and formula materialization
- Implemented a method to remove stale calculation chains in XSSFWorkbook to prevent Excel errors.
- Added functionality to materialize header formulas before shifting columns, ensuring data integrity.
- Updated hours formatting logic to apply consistent styles based on existing cell formats.
- Added unit test to verify the absence of calculation chains after processing.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -165,11 +165,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="56" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
@@ -611,8 +612,8 @@
       <c r="F9" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="J9" t="n" s="4">
-        <v>3.0</v>
+      <c r="J9" t="n" s="5">
+        <v>4.0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -646,8 +647,8 @@
       <c r="F11" t="n" s="0">
         <v>2.0</v>
       </c>
-      <c r="J11" t="n" s="4">
-        <v>4.0</v>
+      <c r="J11" t="n" s="5">
+        <v>6.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor date handling in WbsWorkbook and MainFrame to enforce date column validation
- Updated WbsWorkbook to throw an exception if the date column is missing when writing data, ensuring data integrity.
- Enhanced MainFrame to provide user feedback when attempting to save without a valid date column.
- Modified unit tests to verify that writing operations correctly handle missing date columns, improving error handling.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -613,7 +613,7 @@
         <v>1.0</v>
       </c>
       <c r="J9" t="n" s="5">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -648,7 +648,7 @@
         <v>2.0</v>
       </c>
       <c r="J11" t="n" s="5">
-        <v>6.0</v>
+        <v>4.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement backup functionality in WbsWorkbook save method
- Enhanced the save method in WbsWorkbook to create a timestamped backup of the existing file before overwriting it.
- Updated MainFrame to display a message indicating the backup file path after a successful save.
- Added a unit test to verify the creation of the backup file with the correct naming convention and location.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -165,11 +165,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="56" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
@@ -615,6 +616,9 @@
       <c r="J9" t="n" s="5">
         <v>3.0</v>
       </c>
+      <c r="K9" s="6" t="n">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="0">
@@ -649,6 +653,9 @@
       </c>
       <c r="J11" t="n" s="5">
         <v>4.0</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>2.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement application settings management and enhance backup functionality
- Introduced AppSettings class to manage application settings stored in a properties file, replacing the previous Preferences approach.
- Updated LayoutConfig to load and save settings using the new AppSettings class, improving configuration management.
- Refactored WbsWorkbook and MainFrame to utilize AppSettings for backup directory and last used file paths.
- Enhanced MainFrame UI with a row header for better data visibility and user interaction.
- Added unit tests for AppSettings to ensure correct loading and saving of properties.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileSharing readOnlyRecommended="1"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n-sug.INSPIRON5515\Desktop\github\excel-edit-java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8A1DC53-3993-4461-B410-69CCC9D5121A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7062C80-7C67-4684-BF2C-76532CFF7158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4995" yWindow="1215" windowWidth="22065" windowHeight="13215" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +17,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="true"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -165,14 +165,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="56" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -459,48 +457,42 @@
     <col min="1" max="1" bestFit="true" customWidth="true" width="6.0"/>
     <col min="2" max="2" style="1" width="9.0"/>
     <col min="6" max="6" customWidth="true" width="12.0"/>
-    <col min="7" max="7" customWidth="true" width="8.0"/>
-    <col min="8" max="8" customWidth="true" width="8.0"/>
-    <col min="9" max="9" customWidth="true" width="8.0"/>
-    <col min="10" max="10" customWidth="true" width="8.0"/>
-    <col min="11" max="11" customWidth="true" width="8.0"/>
-    <col min="12" max="12" customWidth="true" width="8.0"/>
-    <col min="13" max="13" customWidth="true" width="8.0"/>
+    <col min="7" max="13" customWidth="true" width="8.0"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="F2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="G2" s="3">
         <v>46296</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="3">
         <f t="shared" ref="H2:M2" si="0">G2+1</f>
-        <v>46297.0</v>
-      </c>
-      <c r="I2" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="I2" s="3">
         <f t="shared" si="0"/>
-        <v>46298.0</v>
-      </c>
-      <c r="J2" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="J2" s="3">
         <f t="shared" si="0"/>
-        <v>46299.0</v>
-      </c>
-      <c r="K2" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="K2" s="3">
         <f t="shared" si="0"/>
-        <v>46300.0</v>
-      </c>
-      <c r="L2" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L2" s="3">
         <f t="shared" si="0"/>
-        <v>46301.0</v>
-      </c>
-      <c r="M2" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="M2" s="3">
         <f t="shared" si="0"/>
-        <v>46302.0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" t="s" s="0">
         <v>1</v>
       </c>
@@ -542,7 +534,7 @@
         <v>水</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:13">
       <c r="A4" s="0">
         <v>1</v>
       </c>
@@ -556,13 +548,13 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:13">
       <c r="D5" s="2"/>
       <c r="E5" t="s" s="0">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:13">
       <c r="A6" s="0">
         <v>2</v>
       </c>
@@ -576,13 +568,13 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:13">
       <c r="D7" s="2"/>
       <c r="E7" t="s" s="0">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:13">
       <c r="A8" s="0">
         <v>3</v>
       </c>
@@ -598,11 +590,8 @@
       <c r="E8" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="J8" t="n" s="0">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+    </row>
+    <row r="9" spans="1:13">
       <c r="D9" s="2" t="str">
         <f>D8</f>
         <v>菅原</v>
@@ -610,17 +599,15 @@
       <c r="E9" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="F9" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="J9" t="n" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+      <c r="F9" s="0">
+        <v>1</v>
+      </c>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4" t="n">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="0">
         <v>3</v>
       </c>
@@ -636,11 +623,8 @@
       <c r="E10" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="J10" t="n" s="0">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+    </row>
+    <row r="11" spans="1:13">
       <c r="D11" s="2" t="str">
         <f>D10</f>
         <v>菅原</v>
@@ -648,14 +632,12 @@
       <c r="E11" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="F11" t="n" s="0">
-        <v>2.0</v>
-      </c>
-      <c r="J11" t="n" s="5">
-        <v>4.0</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>2.0</v>
+      <c r="F11" s="0">
+        <v>2</v>
+      </c>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4" t="n">
+        <v>5.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance filtering functionality in WbsFilter and MainFrame
- Updated WbsFilter to include an option for filtering WbsItems based on actual entries, allowing users to view only items with recorded actuals.
- Modified MainFrame to add a checkbox for the "実績ありのみ" filter, improving user interface and experience.
- Refactored file loading and filtering logic to accommodate the new filtering option.
- Updated README.md to reflect changes in usage instructions for loading Excel files and applying filters.
- Added unit tests to verify the new filtering behavior and ensure correct functionality.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -9,7 +9,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n-sug.INSPIRON5515\Desktop\github\excel-edit-java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7062C80-7C67-4684-BF2C-76532CFF7158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC1F2DB-21E4-405A-B2CB-FFB1983831BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4995" yWindow="1215" windowWidth="22065" windowHeight="13215" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
   <si>
     <t>WBS No</t>
     <phoneticPr fontId="1"/>
@@ -564,6 +564,9 @@
       <c r="C6" t="s" s="0">
         <v>4</v>
       </c>
+      <c r="D6" t="s" s="0">
+        <v>6</v>
+      </c>
       <c r="E6" t="s" s="0">
         <v>7</v>
       </c>
@@ -603,8 +606,8 @@
         <v>1</v>
       </c>
       <c r="J9" s="4"/>
-      <c r="K9" s="4" t="n">
-        <v>5.0</v>
+      <c r="K9" s="4">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -636,9 +639,7 @@
         <v>2</v>
       </c>
       <c r="J11" s="4"/>
-      <c r="K11" s="4" t="n">
-        <v>5.0</v>
-      </c>
+      <c r="K11" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>

<commit_message>
Implement file modification detection and UI updates in WbsWorkbook and MainFrame
- Enhanced WbsWorkbook to detect external modifications to the file after loading, throwing a ConcurrentFileChangeException if changes are detected, ensuring data integrity.
- Updated MainFrame to display file information, including whether the workbook is a legacy shared workbook and the last modified time, improving user awareness.
- Modified README.md to include new error handling instructions for file modifications and updated UI information.
- Added unit tests to validate the new file modification detection and ensure correct behavior during save operations.
</commit_message>
<xml_diff>
--- a/wbs_sample.xlsx
+++ b/wbs_sample.xlsx
@@ -4,21 +4,24 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <fileSharing readOnlyRecommended="1"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n-sug.INSPIRON5515\Desktop\github\excel-edit-java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC1F2DB-21E4-405A-B2CB-FFB1983831BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{60A9669C-E92E-48C3-8FCA-C9FA6DB1AD66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4995" yWindow="1215" windowWidth="22065" windowHeight="13215" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="2115" windowWidth="22065" windowHeight="12435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="true"/>
+  <calcPr calcId="191029"/>
+  <customWorkbookViews>
+    <customWorkbookView name="菅原規司 - 個人用ビュー" guid="{21E44BE2-B3BD-4D6E-9054-A55450FB801F}" mergeInterval="0" personalView="1" xWindow="430" yWindow="184" windowWidth="1471" windowHeight="829" activeSheetId="1"/>
+  </customWorkbookViews>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -121,7 +124,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -186,6 +188,54 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{61DE16DC-477D-4FCD-B5A1-DDDD5EEDF634}" diskRevisions="1" revisionId="2" version="3">
+  <header guid="{0D429DB6-8EC4-4832-B3E9-B82E9AA9A7EE}" dateTime="2026-10-06T07:50:14" maxSheetId="2" userName="菅原規司" r:id="rId1">
+    <sheetIdMap count="1">
+      <sheetId val="1"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{8AED5371-E01B-4EDE-9427-9B732F9CF87D}" dateTime="2026-10-06T07:51:16" maxSheetId="2" userName="菅原規司" r:id="rId2" minRId="1">
+    <sheetIdMap count="1">
+      <sheetId val="1"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{61DE16DC-477D-4FCD-B5A1-DDDD5EEDF634}" dateTime="2026-10-06T07:53:44" maxSheetId="2" userName="菅原規司" r:id="rId3" minRId="2">
+    <sheetIdMap count="1">
+      <sheetId val="1"/>
+    </sheetIdMap>
+  </header>
+</headers>
+</file>
+
+<file path=xl/revisions/revisionLog1.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac"/>
+</file>
+
+<file path=xl/revisions/revisionLog2.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="1" sId="1">
+    <nc r="L9">
+      <v>5</v>
+    </nc>
+  </rcc>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog3.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="2" sId="1" numFmtId="4">
+    <nc r="K11">
+      <v>3</v>
+    </nc>
+  </rcc>
+</revisions>
+</file>
+
+<file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -454,14 +504,14 @@
   <dimension ref="A2:M11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="6.0"/>
-    <col min="2" max="2" style="1" width="9.0"/>
-    <col min="6" max="6" customWidth="true" width="12.0"/>
-    <col min="7" max="13" customWidth="true" width="8.0"/>
+    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:13">
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="3">
@@ -493,104 +543,104 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" t="s" s="0">
+      <c r="F3" t="s">
         <v>13</v>
       </c>
-      <c r="G3" t="str" s="0">
+      <c r="G3" t="str">
         <f>TEXT(G2,"aaa")</f>
         <v>木</v>
       </c>
-      <c r="H3" t="str" s="0">
+      <c r="H3" t="str">
         <f t="shared" ref="H3:M3" si="1">TEXT(H2,"aaa")</f>
         <v>金</v>
       </c>
-      <c r="I3" t="str" s="0">
+      <c r="I3" t="str">
         <f t="shared" si="1"/>
         <v>土</v>
       </c>
-      <c r="J3" t="str" s="0">
+      <c r="J3" t="str">
         <f t="shared" si="1"/>
         <v>日</v>
       </c>
-      <c r="K3" t="str" s="0">
+      <c r="K3" t="str">
         <f t="shared" si="1"/>
         <v>月</v>
       </c>
-      <c r="L3" t="str" s="0">
+      <c r="L3" t="str">
         <f t="shared" si="1"/>
         <v>火</v>
       </c>
-      <c r="M3" t="str" s="0">
+      <c r="M3" t="str">
         <f t="shared" si="1"/>
         <v>水</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="0">
+      <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="E4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="D5" s="2"/>
-      <c r="E5" t="s" s="0">
+      <c r="E5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="0">
+      <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="D6" t="s">
         <v>6</v>
       </c>
-      <c r="E6" t="s" s="0">
+      <c r="E6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="D7" s="2"/>
-      <c r="E7" t="s" s="0">
+      <c r="E7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="0">
+      <c r="A8">
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="C8" t="s">
         <v>10</v>
       </c>
-      <c r="D8" t="s" s="0">
+      <c r="D8" t="s">
         <v>6</v>
       </c>
-      <c r="E8" t="s" s="0">
+      <c r="E8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -599,31 +649,34 @@
         <f>D8</f>
         <v>菅原</v>
       </c>
-      <c r="E9" t="s" s="0">
+      <c r="E9" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="0">
+      <c r="F9">
         <v>1</v>
       </c>
       <c r="J9" s="4"/>
       <c r="K9" s="4">
         <v>5</v>
       </c>
+      <c r="L9">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="0">
+      <c r="A10">
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" t="s" s="0">
+      <c r="C10" t="s">
         <v>11</v>
       </c>
-      <c r="D10" t="s" s="0">
+      <c r="D10" t="s">
         <v>6</v>
       </c>
-      <c r="E10" t="s" s="0">
+      <c r="E10" t="s">
         <v>7</v>
       </c>
     </row>
@@ -632,16 +685,25 @@
         <f>D10</f>
         <v>菅原</v>
       </c>
-      <c r="E11" t="s" s="0">
+      <c r="E11" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="0">
+      <c r="F11">
         <v>2</v>
       </c>
       <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
+      <c r="K11" s="4">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
+  <customSheetViews>
+    <customSheetView guid="{21E44BE2-B3BD-4D6E-9054-A55450FB801F}">
+      <pane ySplit="3" topLeftCell="A4" activePane="bottomLeft" state="frozen"/>
+      <selection pane="bottomLeft" activeCell="D6" sqref="D6"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+    </customSheetView>
+  </customSheetViews>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>